<commit_message>
Add draft Telugu translations for the 4 WhatsApp notice templates
Filled in the "TBD" Telugu rows in automation/whatsapp-templates.md
(hearing, show_cause, closure, order) at the user's request, resolving
the "are notices bilingual" open decision as yes.

Important: these are AI-assisted draft translations, not reviewed by
a native Telugu speaker. Marked with an explicit warning under each
one - do not submit to Meta or send to a real party until departmental
staff with strong Telugu review them line by line. Flagged specific
terms worth extra scrutiny (ex-parte, show cause, compliance, the
office designation in the footer). Act names and dates are kept
unchanged from the English version rather than translated, matching
how Indian regional-language legal notices conventionally cite Acts.

Updated CLAUDE.md and the Excel plan's Overview tab (open decisions)
to record this as decided-but-unreviewed, not silently resolved.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Labour_Portal_Full_Development_Plan.xlsx
+++ b/Labour_Portal_Full_Development_Plan.xlsx
@@ -708,7 +708,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>1) Can staff see their own slice of the Monthly MIS?  2) Are notices bilingual (Telugu + English)?  3) Is file_number unique per office (multi-office) or statewide?  4) PDF output needed, or DOCX only?  5) Owners for each Roadmap task</t>
+          <t>1) Can staff see their own slice of the Monthly MIS?  2) Telugu notices: DECIDED - yes. Draft Telugu WhatsApp templates exist (automation/whatsapp-templates.md) but are AI-assisted and unreviewed - a native Telugu speaker on staff must check them before Meta submission or real use. The DOCX letterhead templates still need real Telugu content once drafted.  3) Is file_number unique per office (multi-office) or statewide?  4) PDF output needed, or DOCX only?  5) Owners for each Roadmap task</t>
         </is>
       </c>
     </row>
@@ -4659,8 +4659,8 @@
   <mergeCells count="14">
     <mergeCell ref="A5:A23"/>
     <mergeCell ref="A52:A62"/>
+    <mergeCell ref="A70:A75"/>
     <mergeCell ref="A40:A51"/>
-    <mergeCell ref="A70:A75"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A24:A32"/>
     <mergeCell ref="A87:A91"/>

</xml_diff>